<commit_message>
gui eklendi bazı hatalar düzeltildi (hala eksikleri vardır)
</commit_message>
<xml_diff>
--- a/sinav_programi.xlsx
+++ b/sinav_programi.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13.10.2025</t>
+          <t>17.10.2025</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -468,1089 +468,1043 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BLM449</t>
+          <t>BLM211</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bilgisayarlı Görmenin Temelleri</t>
+          <t>Mantıksal Tasarım ve Uygulamalar</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>Buyuk Amfi, 305, Yiğido</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13.10.2025</t>
+          <t>17.10.2025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEÇİMLİK DERS </t>
+          <t>BLM305</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NaN</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>İşletim Sistemleri</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Buyuk Amfi, 303, 301</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13.10.2025</t>
+          <t>17.10.2025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEÇMELİ DERS </t>
+          <t>TDB107</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NaN</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Türk Dili I</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>301, umut, Buyuk Amfi</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13.10.2025</t>
+          <t>17.10.2025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MUH301</t>
+          <t>BLM417</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sayısal Yöntemler</t>
+          <t>Programlanabilir Yapılar</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>Buyuk Amfi, EDA, 305</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13.10.2025</t>
+          <t>17.10.2025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BLM101</t>
+          <t>BLM401</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bilgisayar Laboratuvarı I</t>
+          <t>Bilgisayar Ağları</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>301, umut, Buyuk Amfi</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13.10.2025</t>
+          <t>17.10.2025</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BLM309</t>
+          <t>BLM421</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Staj II</t>
+          <t>Yazılım Proje Yönetimi</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>301, Yiğido, EDA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13.10.2025</t>
+          <t>20.10.2025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MUH445</t>
+          <t>FEF111</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Mühendisler için İstatistik</t>
+          <t>Fizik I</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>305, Yiğido, umut</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13.10.2025</t>
+          <t>20.10.2025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BLM405</t>
+          <t>BLM323</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>İş Hayatı ve İş Güvenliğine Hazırlık</t>
+          <t>Bilgi Güvenliği ve Kriptografi</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>umut, 303, Yiğido</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>14.10.2025</t>
+          <t>20.10.2025</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BLM103</t>
+          <t>BLM205</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bilgisayar Mühendisliğine Giriş</t>
+          <t>Ayrık Matematik</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>301, umut, Yiğido</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14.10.2025</t>
+          <t>20.10.2025</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BLM321</t>
+          <t>BLM103</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Robotlar için Matematik Temelleri</t>
+          <t>Bilgisayar Mühendisliğine Giriş</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>Buyuk Amfi, Yiğido, umut</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14.10.2025</t>
+          <t>20.10.2025</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FEF203</t>
+          <t>BLM209</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Diferansiyel Denklemler</t>
+          <t xml:space="preserve">Programlama Laboratuvarı - I </t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, 301, Yiğido</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14.10.2025</t>
+          <t>20.10.2025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BLM401</t>
+          <t>BLM213</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Bilgisayar Ağları</t>
+          <t>Staj I</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, umut, 305</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>14.10.2025</t>
+          <t>21.10.2025</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BLM411</t>
+          <t>BLM321</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Bilgisayar Semineri</t>
+          <t>Robotlar için Matematik Temelleri</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>305, umut, 303</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>14.10.2025</t>
+          <t>21.10.2025</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BLM323</t>
+          <t>MUH301</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Bilgi Güvenliği ve Kriptografi</t>
+          <t>Sayısal Yöntemler</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>303, umut, Yiğido</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>21.10.2025</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>FEF111</t>
+          <t>MUH403</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Fizik I</t>
+          <t>Araştırma Problemleri</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>301, Yiğido, 305</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>21.10.2025</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BLM417</t>
+          <t>MUH402</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Programlanabilir Yapılar</t>
+          <t>Bitirme Çalışması</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>umut, Yiğido, 305</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>21.10.2025</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MUH403</t>
+          <t>BLM303</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Araştırma Problemleri</t>
+          <t>İşaret ve Sistemler</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, 301, Buyuk Amfi</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>21.10.2025</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BLM105</t>
+          <t>AIT109</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Programlama I </t>
+          <t>Atatürk İlkeleri ve İnkılap Tarihi I</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, 305, Buyuk Amfi</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>22.10.2025</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TDB107</t>
+          <t>YDB117</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Türk Dili I</t>
+          <t>İngilizce I</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, 305, Buyuk Amfi</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>22.10.2025</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BLM207</t>
+          <t>BLM307</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Veri Yapıları ve Algoritmaları</t>
+          <t xml:space="preserve">Yazılım Laboratuvarı I </t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, 301, 303</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>16.10.2025</t>
+          <t>22.10.2025</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BLM451</t>
+          <t>BLM207</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Derin Öğrenmenin Temelleri</t>
+          <t>Veri Yapıları ve Algoritmaları</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>umut, Buyuk Amfi, 301</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>16.10.2025</t>
+          <t>22.10.2025</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BLM441</t>
+          <t>FEF203</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mobil Programlama</t>
+          <t>Diferansiyel Denklemler</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>303, Buyuk Amfi, umut</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>16.10.2025</t>
+          <t>22.10.2025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BLM443</t>
+          <t>BLM451</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Doğal Dil İşleme ve Metin Madenciliğine Giriş</t>
+          <t>Derin Öğrenmenin Temelleri</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>305, EDA, Buyuk Amfi</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>16.10.2025</t>
+          <t>22.10.2025</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>YDB117</t>
+          <t>BLM429</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>İngilizce I</t>
+          <t>Veri Madenciliğine Giriş</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, Buyuk Amfi, 303</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>16.10.2025</t>
+          <t>23.10.2025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FEF115</t>
+          <t>BLM411</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Matematik I</t>
+          <t>Bilgisayar Semineri</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, umut, 301</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16.10.2025</t>
+          <t>23.10.2025</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BLM209</t>
+          <t>MUH413</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Programlama Laboratuvarı - I </t>
+          <t>Gezgin Robotlara Giriş</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, umut, 301</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>17.10.2025</t>
+          <t>23.10.2025</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BLM307</t>
+          <t>BLM449</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yazılım Laboratuvarı I </t>
+          <t>Bilgisayarlı Görmenin Temelleri</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>Yiğido, EDA, umut</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>17.10.2025</t>
+          <t>23.10.2025</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MUH402</t>
+          <t>MUH201</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Bitirme Çalışması</t>
+          <t>Nesneye Yönelik Programlama</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>Yiğido, umut, 305</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>17.10.2025</t>
+          <t>23.10.2025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>BLM435</t>
+          <t>BLM325</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Biyoinformatiğe Giriş</t>
+          <t>Mikroişlemci Sistemleri</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>umut, Yiğido, Buyuk Amfi</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>17.10.2025</t>
+          <t>23.10.2025</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BLM303</t>
+          <t>BLM101</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>İşaret ve Sistemler</t>
+          <t>Bilgisayar Laboratuvarı I</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>305, 301, 303</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MUH413</t>
+          <t>BLM309</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Gezgin Robotlara Giriş</t>
+          <t>Staj II</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>EDA, 303, 305</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>17.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AIT109</t>
+          <t>FEF113</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Atatürk İlkeleri ve İnkılap Tarihi I</t>
+          <t>Lineer Cebir</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>umut, EDA, Yiğido</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>20.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>BLM205</t>
+          <t>BLM405</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Ayrık Matematik</t>
+          <t>İş Hayatı ve İş Güvenliğine Hazırlık</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>303, Yiğido, umut</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>BLM429</t>
+          <t>FEF115</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Veri Madenciliğine Giriş</t>
+          <t>Matematik I</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>301, EDA, 305</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>20.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>BLM213</t>
+          <t>MUH445</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Staj I</t>
+          <t>Mühendisler için İstatistik</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>305, Buyuk Amfi, EDA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>20.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>BLM211</t>
+          <t>BLM443</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mantıksal Tasarım ve Uygulamalar</t>
+          <t>Doğal Dil İşleme ve Metin Madenciliğine Giriş</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>umut, 303, Yiğido</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>20.10.2025</t>
+          <t>27.10.2025</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FEF113</t>
+          <t>BLM435</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Lineer Cebir</t>
+          <t>Biyoinformatiğe Giriş</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>303, EDA, Buyuk Amfi</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>20.10.2025</t>
+          <t>27.10.2025</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>BLM325</t>
+          <t>BLM105</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mikroişlemci Sistemleri</t>
+          <t xml:space="preserve">Programlama I </t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>305, umut, Yiğido</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>21.10.2025</t>
+          <t>27.10.2025</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>BLM421</t>
+          <t>BLM441</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Yazılım Proje Yönetimi</t>
+          <t>Mobil Programlama</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Buyuk Amfi, 301, 305</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>21.10.2025</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>BLM305</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>İşletim Sistemleri</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Buyuk Amfi, 301, 305</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>21.10.2025</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>MUH201</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Nesneye Yönelik Programlama</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Buyuk Amfi, 301, 305</t>
+          <t>301, Buyuk Amfi, 305</t>
         </is>
       </c>
     </row>

</xml_diff>